<commit_message>
Fill campaign templates with transcribed dialogue
The sheet used placeholders ("Candidate speaks", "none") instead of real
lines for 7 templates. Their videos have audio, so transcribe each and bake
the dialogue into the templates, keeping the intro/outro screens:
Maine Candidate 6, Save the Day 22, Chicken Little 7, Cheeseburger Fail 10,
Korea Rain 7, Buried Alive 2. Bollywood Action stays empty (no speech in the
video). Speaker labels are generic (Speaker 1/2) — rename in the studio.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/subtitles/campaign-2026.xlsx
+++ b/templates/subtitles/campaign-2026.xlsx
@@ -65,8 +65,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -398,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K76"/>
+  <dimension ref="A1:K123"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -716,131 +717,149 @@
       <c r="C17" t="str">
         <v>maine candidate</v>
       </c>
-      <c r="D17" t="str">
-        <v>:00</v>
-      </c>
-      <c r="E17" t="str">
-        <v>:45</v>
+      <c r="D17" s="1">
+        <v>0</v>
+      </c>
+      <c r="E17" s="1">
+        <v>0.000038657407407407404</v>
       </c>
       <c r="F17" t="str">
-        <v>Ashley Webb</v>
+        <v>Speaker 1</v>
       </c>
       <c r="G17" t="str">
-        <v>(Candidate speaks)</v>
+        <v>Ashley Webb, what qualifications do you have to serve in the U.S.</v>
+      </c>
+      <c r="H17">
+        <v>65</v>
       </c>
     </row>
     <row r="18">
       <c r="A18">
         <v>0</v>
       </c>
-      <c r="D18" t="str">
-        <v>outro</v>
-      </c>
-      <c r="E18" t="str">
-        <v>outro</v>
+      <c r="C18" t="str">
+        <v>maine candidate</v>
+      </c>
+      <c r="D18" s="1">
+        <v>0.00004027777777777778</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0.00004074074074074074</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Speaker 2</v>
       </c>
       <c r="G18" t="str">
-        <v>Vote for [Candidate X] on November 3</v>
+        <v>Senate?</v>
+      </c>
+      <c r="H18">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>0</v>
+      </c>
+      <c r="C19" t="str">
+        <v>maine candidate</v>
+      </c>
+      <c r="D19" s="1">
+        <v>0.000049768518518518516</v>
+      </c>
+      <c r="E19" s="1">
+        <v>0.00007638888888888889</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Speaker 1</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Oh, I ran for office several times.</v>
+      </c>
+      <c r="H19">
+        <v>35</v>
       </c>
     </row>
     <row r="20">
       <c r="A20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C20" t="str">
-        <v>voter id</v>
-      </c>
-      <c r="D20" t="str">
-        <v>title</v>
-      </c>
-      <c r="E20" t="str">
-        <v>title</v>
+        <v>maine candidate</v>
+      </c>
+      <c r="D20" s="1">
+        <v>0.00007777777777777778</v>
+      </c>
+      <c r="E20" s="1">
+        <v>0.00009837962962962963</v>
       </c>
       <c r="F20" t="str">
-        <v>meta data</v>
+        <v>Speaker 1</v>
       </c>
       <c r="G20" t="str">
-        <v>Who are the real election deniers?</v>
+        <v>Didn't win, but I did run.</v>
+      </c>
+      <c r="H20">
+        <v>26</v>
       </c>
     </row>
     <row r="21">
       <c r="A21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C21" t="str">
-        <v>voter id</v>
-      </c>
-      <c r="D21" t="str">
-        <v>description</v>
-      </c>
-      <c r="E21" t="str">
-        <v>description</v>
+        <v>maine candidate</v>
+      </c>
+      <c r="D21" s="1">
+        <v>0.00010023148148148148</v>
+      </c>
+      <c r="E21" s="1">
+        <v>0.00019328703703703703</v>
       </c>
       <c r="F21" t="str">
-        <v>meta data</v>
+        <v>Speaker 1</v>
       </c>
       <c r="G21" t="str">
-        <v>A battle over voter ID breaks out in a reimagined court scene from a South Asian drama.</v>
+        <v>And then I'm a songwriter and then I write my own books and then I suppose my transparency.</v>
+      </c>
+      <c r="H21">
+        <v>91</v>
       </c>
     </row>
     <row r="22">
       <c r="A22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C22" t="str">
-        <v>voter id</v>
-      </c>
-      <c r="D22" t="str">
-        <v>:00</v>
-      </c>
-      <c r="E22" t="str">
-        <v>:02</v>
+        <v>maine candidate</v>
+      </c>
+      <c r="D22" s="1">
+        <v>0.00020069444444444445</v>
+      </c>
+      <c r="E22" s="1">
+        <v>0.000256712962962963</v>
       </c>
       <c r="F22" t="str">
-        <v>counsel</v>
+        <v>Speaker 1</v>
       </c>
       <c r="G22" t="str">
-        <v>Requiring an ID to vote is racist!</v>
+        <v>I wouldn't lie to the people and I wouldn't deceive the people like we're being deceived right now.</v>
+      </c>
+      <c r="H22">
+        <v>99</v>
       </c>
     </row>
     <row r="23">
       <c r="A23">
-        <v>1</v>
-      </c>
-      <c r="C23" t="str">
-        <v>voter id</v>
+        <v>0</v>
       </c>
       <c r="D23" t="str">
-        <v>:03</v>
+        <v>outro</v>
       </c>
       <c r="E23" t="str">
-        <v>:06</v>
-      </c>
-      <c r="F23" t="str">
-        <v>judge</v>
+        <v>outro</v>
       </c>
       <c r="G23" t="str">
-        <v>Hey? You must explain your position.</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24">
-        <v>1</v>
-      </c>
-      <c r="C24" t="str">
-        <v>voter id</v>
-      </c>
-      <c r="D24" t="str">
-        <v>:08</v>
-      </c>
-      <c r="E24" t="str">
-        <v>:09</v>
-      </c>
-      <c r="F24" t="str">
-        <v>plaintiff</v>
-      </c>
-      <c r="G24" t="str">
-        <v>My dear mother is an example.</v>
+        <v>Vote for [Candidate X] on November 3</v>
       </c>
     </row>
     <row r="25">
@@ -851,16 +870,16 @@
         <v>voter id</v>
       </c>
       <c r="D25" t="str">
-        <v>:09</v>
+        <v>title</v>
       </c>
       <c r="E25" t="str">
-        <v>:10</v>
+        <v>title</v>
       </c>
       <c r="F25" t="str">
-        <v>judge</v>
+        <v>meta data</v>
       </c>
       <c r="G25" t="str">
-        <v>That is so?</v>
+        <v>Who are the real election deniers?</v>
       </c>
     </row>
     <row r="26">
@@ -871,16 +890,16 @@
         <v>voter id</v>
       </c>
       <c r="D26" t="str">
-        <v>:10</v>
+        <v>description</v>
       </c>
       <c r="E26" t="str">
-        <v>:11</v>
+        <v>description</v>
       </c>
       <c r="F26" t="str">
-        <v>plaintiff</v>
+        <v>meta data</v>
       </c>
       <c r="G26" t="str">
-        <v>She has no one to take her to the DMV.</v>
+        <v>A battle over voter ID breaks out in a reimagined court scene from a South Asian drama.</v>
       </c>
     </row>
     <row r="27">
@@ -891,16 +910,16 @@
         <v>voter id</v>
       </c>
       <c r="D27" t="str">
-        <v>:11</v>
+        <v>:00</v>
       </c>
       <c r="E27" t="str">
-        <v>:15</v>
+        <v>:02</v>
       </c>
       <c r="F27" t="str">
-        <v>judge</v>
+        <v>counsel</v>
       </c>
       <c r="G27" t="str">
-        <v>Why don't you take her? She can get a photo ID without cost!</v>
+        <v>Requiring an ID to vote is racist!</v>
       </c>
     </row>
     <row r="28">
@@ -911,16 +930,16 @@
         <v>voter id</v>
       </c>
       <c r="D28" t="str">
-        <v>:15</v>
+        <v>:03</v>
       </c>
       <c r="E28" t="str">
-        <v>:16</v>
+        <v>:06</v>
       </c>
       <c r="F28" t="str">
-        <v>counsel</v>
+        <v>judge</v>
       </c>
       <c r="G28" t="str">
-        <v>No.</v>
+        <v>Hey? You must explain your position.</v>
       </c>
     </row>
     <row r="29">
@@ -931,16 +950,16 @@
         <v>voter id</v>
       </c>
       <c r="D29" t="str">
-        <v>:17</v>
+        <v>:08</v>
       </c>
       <c r="E29" t="str">
-        <v>:22</v>
+        <v>:09</v>
       </c>
       <c r="F29" t="str">
-        <v>judge</v>
+        <v>plaintiff</v>
       </c>
       <c r="G29" t="str">
-        <v>No? There is nothing preventing her from getting one.</v>
+        <v>My dear mother is an example.</v>
       </c>
     </row>
     <row r="30">
@@ -951,16 +970,16 @@
         <v>voter id</v>
       </c>
       <c r="D30" t="str">
-        <v>:23</v>
+        <v>:09</v>
       </c>
       <c r="E30" t="str">
-        <v>:25</v>
+        <v>:10</v>
       </c>
       <c r="F30" t="str">
-        <v>counsel</v>
+        <v>judge</v>
       </c>
       <c r="G30" t="str">
-        <v>But what if her bursitis flares up?</v>
+        <v>That is so?</v>
       </c>
     </row>
     <row r="31">
@@ -971,16 +990,16 @@
         <v>voter id</v>
       </c>
       <c r="D31" t="str">
-        <v>:26</v>
+        <v>:10</v>
       </c>
       <c r="E31" t="str">
-        <v>:28</v>
+        <v>:11</v>
       </c>
       <c r="F31" t="str">
-        <v>judge</v>
+        <v>plaintiff</v>
       </c>
       <c r="G31" t="str">
-        <v>You Democrats are making yourselves very clear now.</v>
+        <v>She has no one to take her to the DMV.</v>
       </c>
     </row>
     <row r="32">
@@ -991,16 +1010,16 @@
         <v>voter id</v>
       </c>
       <c r="D32" t="str">
-        <v>:29</v>
+        <v>:11</v>
       </c>
       <c r="E32" t="str">
-        <v>:33</v>
+        <v>:15</v>
       </c>
       <c r="F32" t="str">
         <v>judge</v>
       </c>
       <c r="G32" t="str">
-        <v>It's not Donald Trump who wants to end elections.</v>
+        <v>Why don't you take her? She can get a photo ID without cost!</v>
       </c>
     </row>
     <row r="33">
@@ -1011,16 +1030,16 @@
         <v>voter id</v>
       </c>
       <c r="D33" t="str">
-        <v>outro</v>
+        <v>:15</v>
       </c>
       <c r="E33" t="str">
-        <v>outro</v>
+        <v>:16</v>
       </c>
       <c r="F33" t="str">
-        <v>black screen</v>
+        <v>counsel</v>
       </c>
       <c r="G33" t="str">
-        <v>Protect your vote</v>
+        <v>No.</v>
       </c>
     </row>
     <row r="34">
@@ -1031,79 +1050,105 @@
         <v>voter id</v>
       </c>
       <c r="D34" t="str">
-        <v>outro</v>
+        <v>:17</v>
       </c>
       <c r="E34" t="str">
-        <v>outro</v>
+        <v>:22</v>
       </c>
       <c r="F34" t="str">
-        <v>black screen</v>
+        <v>judge</v>
       </c>
       <c r="G34" t="str">
-        <v>Vote for Republican  [Candidate X] on November 3</v>
+        <v>No? There is nothing preventing her from getting one.</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="str">
+        <v>voter id</v>
+      </c>
+      <c r="D35" t="str">
+        <v>:23</v>
+      </c>
+      <c r="E35" t="str">
+        <v>:25</v>
+      </c>
+      <c r="F35" t="str">
+        <v>counsel</v>
+      </c>
+      <c r="G35" t="str">
+        <v>But what if her bursitis flares up?</v>
       </c>
     </row>
     <row r="36">
       <c r="A36">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C36" t="str">
-        <v>bollywood action</v>
+        <v>voter id</v>
       </c>
       <c r="D36" t="str">
-        <v>title</v>
+        <v>:26</v>
       </c>
       <c r="E36" t="str">
-        <v>title</v>
+        <v>:28</v>
       </c>
       <c r="F36" t="str">
-        <v>meta data</v>
+        <v>judge</v>
       </c>
       <c r="G36" t="str">
-        <v>Law enforcement you can count on.</v>
+        <v>You Democrats are making yourselves very clear now.</v>
       </c>
     </row>
     <row r="37">
       <c r="A37">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C37" t="str">
-        <v>bollywood action</v>
+        <v>voter id</v>
       </c>
       <c r="D37" t="str">
-        <v>description</v>
+        <v>:29</v>
       </c>
       <c r="E37" t="str">
-        <v>description</v>
+        <v>:33</v>
       </c>
       <c r="F37" t="str">
-        <v>meta data</v>
+        <v>judge</v>
       </c>
       <c r="G37" t="str">
-        <v>A law-enforcement officer goes to extraordinary, against-all-odds lengths to protect his citizens.</v>
+        <v>It's not Donald Trump who wants to end elections.</v>
       </c>
     </row>
     <row r="38">
       <c r="A38">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C38" t="str">
-        <v>bollywood action</v>
+        <v>voter id</v>
       </c>
       <c r="D38" t="str">
-        <v>:00</v>
+        <v>outro</v>
       </c>
       <c r="E38" t="str">
-        <v>:38</v>
+        <v>outro</v>
       </c>
       <c r="F38" t="str">
-        <v>Law-enforcement officer (insert Republican candidate's head)</v>
+        <v>black screen</v>
       </c>
       <c r="G38" t="str">
-        <v>none</v>
+        <v>Protect your vote</v>
       </c>
     </row>
     <row r="39">
+      <c r="A39">
+        <v>1</v>
+      </c>
+      <c r="C39" t="str">
+        <v>voter id</v>
+      </c>
       <c r="D39" t="str">
         <v>outro</v>
       </c>
@@ -1114,27 +1159,27 @@
         <v>black screen</v>
       </c>
       <c r="G39" t="str">
-        <v>Safety. Security. Law enforcement you can count on.</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40">
+        <v>Vote for Republican  [Candidate X] on November 3</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41">
         <v>3</v>
       </c>
-      <c r="C40" t="str">
+      <c r="C41" t="str">
         <v>bollywood action</v>
       </c>
-      <c r="D40" t="str">
-        <v>outro</v>
-      </c>
-      <c r="E40" t="str">
-        <v>outro</v>
-      </c>
-      <c r="F40" t="str">
-        <v>black screen</v>
-      </c>
-      <c r="G40" t="str">
-        <v>Vote for Republican  [Candidate X] on November 3</v>
+      <c r="D41" t="str">
+        <v>title</v>
+      </c>
+      <c r="E41" t="str">
+        <v>title</v>
+      </c>
+      <c r="F41" t="str">
+        <v>meta data</v>
+      </c>
+      <c r="G41" t="str">
+        <v>Law enforcement you can count on.</v>
       </c>
     </row>
     <row r="42">
@@ -1142,39 +1187,33 @@
         <v>3</v>
       </c>
       <c r="C42" t="str">
-        <v>buried alive</v>
+        <v>bollywood action</v>
       </c>
       <c r="D42" t="str">
-        <v>title</v>
+        <v>description</v>
       </c>
       <c r="E42" t="str">
-        <v>title</v>
+        <v>description</v>
       </c>
       <c r="F42" t="str">
         <v>meta data</v>
       </c>
       <c r="G42" t="str">
-        <v>Democrats mourn the death of the Constitution</v>
+        <v>A law-enforcement officer goes to extraordinary, against-all-odds lengths to protect his citizens.</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43">
-        <v>3</v>
-      </c>
-      <c r="C43" t="str">
-        <v>buried alive</v>
-      </c>
       <c r="D43" t="str">
-        <v>description</v>
+        <v>outro</v>
       </c>
       <c r="E43" t="str">
-        <v>description</v>
+        <v>outro</v>
       </c>
       <c r="F43" t="str">
-        <v>meta data</v>
+        <v>black screen</v>
       </c>
       <c r="G43" t="str">
-        <v>A burial scene from a Filipino telenovela illustrates what Democrats really think about the Constitution.</v>
+        <v>Safety. Security. Law enforcement you can count on.</v>
       </c>
     </row>
     <row r="44">
@@ -1182,39 +1221,19 @@
         <v>3</v>
       </c>
       <c r="C44" t="str">
-        <v>buried alive</v>
+        <v>bollywood action</v>
       </c>
       <c r="D44" t="str">
-        <v>intro</v>
+        <v>outro</v>
       </c>
       <c r="E44" t="str">
-        <v>intro</v>
+        <v>outro</v>
       </c>
       <c r="F44" t="str">
         <v>black screen</v>
       </c>
       <c r="G44" t="str">
-        <v>Democrats mourn the death of the Constitution</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45">
-        <v>3</v>
-      </c>
-      <c r="C45" t="str">
-        <v>buried alive</v>
-      </c>
-      <c r="D45" t="str">
-        <v>:00</v>
-      </c>
-      <c r="E45" t="str">
-        <v>:19</v>
-      </c>
-      <c r="F45" t="str">
-        <v>Fake mourner</v>
-      </c>
-      <c r="G45" t="str">
-        <v>no added text</v>
+        <v>Vote for Republican  [Candidate X] on November 3</v>
       </c>
     </row>
     <row r="46">
@@ -1225,16 +1244,16 @@
         <v>buried alive</v>
       </c>
       <c r="D46" t="str">
-        <v>outro</v>
+        <v>title</v>
       </c>
       <c r="E46" t="str">
-        <v>outro</v>
+        <v>title</v>
       </c>
       <c r="F46" t="str">
-        <v>black screen</v>
+        <v>meta data</v>
       </c>
       <c r="G46" t="str">
-        <v>Vote like your life depends on it.</v>
+        <v>Democrats mourn the death of the Constitution</v>
       </c>
     </row>
     <row r="47">
@@ -1245,113 +1264,122 @@
         <v>buried alive</v>
       </c>
       <c r="D47" t="str">
-        <v>outro</v>
+        <v>description</v>
       </c>
       <c r="E47" t="str">
-        <v>outro</v>
+        <v>description</v>
       </c>
       <c r="F47" t="str">
+        <v>meta data</v>
+      </c>
+      <c r="G47" t="str">
+        <v>A burial scene from a Filipino telenovela illustrates what Democrats really think about the Constitution.</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48">
+        <v>3</v>
+      </c>
+      <c r="C48" t="str">
+        <v>buried alive</v>
+      </c>
+      <c r="D48" t="str">
+        <v>intro</v>
+      </c>
+      <c r="E48" t="str">
+        <v>intro</v>
+      </c>
+      <c r="F48" t="str">
         <v>black screen</v>
       </c>
-      <c r="G47" t="str">
-        <v>Vote for Republican  [Candidate X] on November 3</v>
+      <c r="G48" t="str">
+        <v>Democrats mourn the death of the Constitution</v>
       </c>
     </row>
     <row r="49">
       <c r="A49">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C49" t="str">
-        <v>save the day</v>
-      </c>
-      <c r="D49" t="str">
-        <v>title</v>
-      </c>
-      <c r="E49" t="str">
-        <v>title</v>
+        <v>buried alive</v>
+      </c>
+      <c r="D49" s="1">
+        <v>0.0001480324074074074</v>
+      </c>
+      <c r="E49" s="1">
+        <v>0.00016099537037037037</v>
       </c>
       <c r="F49" t="str">
-        <v>meta data</v>
+        <v>Speaker 1</v>
       </c>
       <c r="G49" t="str">
-        <v>There's one thing that Democrats and Republicans can agree on.</v>
+        <v>Don't stop!</v>
+      </c>
+      <c r="H49">
+        <v>11</v>
       </c>
     </row>
     <row r="50">
       <c r="A50">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C50" t="str">
-        <v>save the day</v>
-      </c>
-      <c r="D50" t="str">
-        <v>description</v>
-      </c>
-      <c r="E50" t="str">
-        <v>description</v>
+        <v>buried alive</v>
+      </c>
+      <c r="D50" s="1">
+        <v>0.00016724537037037036</v>
+      </c>
+      <c r="E50" s="1">
+        <v>0.0001744212962962963</v>
       </c>
       <c r="F50" t="str">
-        <v>meta data</v>
+        <v>Speaker 2</v>
       </c>
       <c r="G50" t="str">
-        <v>An ad in the Democrats'  famous 2016 Save the Day campaign is reworked for the 2026 midterms</v>
+        <v>Go on!</v>
+      </c>
+      <c r="H50">
+        <v>6</v>
       </c>
     </row>
     <row r="51">
       <c r="A51">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C51" t="str">
-        <v>save the day</v>
+        <v>buried alive</v>
       </c>
       <c r="D51" t="str">
-        <v>intro</v>
+        <v>outro</v>
       </c>
       <c r="E51" t="str">
-        <v>intro</v>
+        <v>outro</v>
       </c>
       <c r="F51" t="str">
         <v>black screen</v>
       </c>
       <c r="G51" t="str">
-        <v>Democrats are right for once …</v>
+        <v>Vote like your life depends on it.</v>
       </c>
     </row>
     <row r="52">
       <c r="A52">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C52" t="str">
-        <v>save the day</v>
+        <v>buried alive</v>
       </c>
       <c r="D52" t="str">
-        <v>:00</v>
+        <v>outro</v>
       </c>
       <c r="E52" t="str">
-        <v>:30</v>
+        <v>outro</v>
+      </c>
+      <c r="F52" t="str">
+        <v>black screen</v>
       </c>
       <c r="G52" t="str">
-        <v>Democrat celebs speak</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53">
-        <v>0</v>
-      </c>
-      <c r="C53" t="str">
-        <v>save the day</v>
-      </c>
-      <c r="D53" t="str">
-        <v>outro</v>
-      </c>
-      <c r="E53" t="str">
-        <v>outro</v>
-      </c>
-      <c r="F53" t="str">
-        <v>black screen</v>
-      </c>
-      <c r="G53" t="str">
-        <v>There's at least one thing we can agree on ...</v>
+        <v>Vote for Republican  [Candidate X] on November 3</v>
       </c>
     </row>
     <row r="54">
@@ -1362,16 +1390,16 @@
         <v>save the day</v>
       </c>
       <c r="D54" t="str">
-        <v>outro</v>
+        <v>title</v>
       </c>
       <c r="E54" t="str">
-        <v>outro</v>
+        <v>title</v>
       </c>
       <c r="F54" t="str">
-        <v>black screen</v>
+        <v>meta data</v>
       </c>
       <c r="G54" t="str">
-        <v>"We cannot pretend both sides are equally unfavorable."</v>
+        <v>There's one thing that Democrats and Republicans can agree on.</v>
       </c>
     </row>
     <row r="55">
@@ -1382,16 +1410,36 @@
         <v>save the day</v>
       </c>
       <c r="D55" t="str">
-        <v>outro</v>
+        <v>description</v>
       </c>
       <c r="E55" t="str">
-        <v>outro</v>
+        <v>description</v>
       </c>
       <c r="F55" t="str">
+        <v>meta data</v>
+      </c>
+      <c r="G55" t="str">
+        <v>An ad in the Democrats'  famous 2016 Save the Day campaign is reworked for the 2026 midterms</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56">
+        <v>0</v>
+      </c>
+      <c r="C56" t="str">
+        <v>save the day</v>
+      </c>
+      <c r="D56" t="str">
+        <v>intro</v>
+      </c>
+      <c r="E56" t="str">
+        <v>intro</v>
+      </c>
+      <c r="F56" t="str">
         <v>black screen</v>
       </c>
-      <c r="G55" t="str">
-        <v>Vote for Republican [Candidate X] on November 3</v>
+      <c r="G56" t="str">
+        <v>Democrats are right for once …</v>
       </c>
     </row>
     <row r="57">
@@ -1399,213 +1447,298 @@
         <v>0</v>
       </c>
       <c r="C57" t="str">
-        <v>chicken little</v>
-      </c>
-      <c r="D57" t="str">
-        <v>title</v>
-      </c>
-      <c r="E57" t="str">
-        <v>title</v>
+        <v>save the day</v>
+      </c>
+      <c r="D57" s="1">
+        <v>0</v>
+      </c>
+      <c r="E57" s="1">
+        <v>0.00002337962962962963</v>
       </c>
       <c r="F57" t="str">
-        <v>meta data</v>
+        <v>Speaker 1</v>
       </c>
       <c r="G57" t="str">
-        <v>The new star of the Democratic Party looks familiar</v>
+        <v>We can save the day.</v>
+      </c>
+      <c r="H57">
+        <v>20</v>
       </c>
     </row>
     <row r="58">
       <c r="A58">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C58" t="str">
-        <v>chicken little</v>
-      </c>
-      <c r="D58" t="str">
-        <v>description</v>
-      </c>
-      <c r="E58" t="str">
-        <v>description</v>
+        <v>save the day</v>
+      </c>
+      <c r="D58" s="1">
+        <v>0.000026157407407407405</v>
+      </c>
+      <c r="E58" s="1">
+        <v>0.00003287037037037037</v>
       </c>
       <c r="F58" t="str">
-        <v>meta data</v>
+        <v>Speaker 1</v>
       </c>
       <c r="G58" t="str">
-        <v>Border walls are useless when the enemy is within, as these clips from the 1943 Disney cartoon Chicken Little illustrate.</v>
+        <v>For our children.</v>
+      </c>
+      <c r="H58">
+        <v>17</v>
       </c>
     </row>
     <row r="59">
       <c r="A59">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C59" t="str">
-        <v>chicken little</v>
-      </c>
-      <c r="D59" t="str">
-        <v>:00</v>
-      </c>
-      <c r="E59">
-        <v>0.041666666666666664</v>
+        <v>save the day</v>
+      </c>
+      <c r="D59" s="1">
+        <v>0.000033796296296296295</v>
+      </c>
+      <c r="E59" s="1">
+        <v>0.00004050925925925926</v>
       </c>
       <c r="F59" t="str">
-        <v>Insert cartoon head of Mamdani on Foxy Loxy</v>
+        <v>Speaker 2</v>
       </c>
       <c r="G59" t="str">
-        <v>cartoon with no text</v>
+        <v>For our children.</v>
+      </c>
+      <c r="H59">
+        <v>17</v>
       </c>
     </row>
     <row r="60">
       <c r="A60">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C60" t="str">
-        <v>chicken little</v>
-      </c>
-      <c r="D60" t="str">
-        <v>outro</v>
-      </c>
-      <c r="E60" t="str">
-        <v>outro</v>
+        <v>save the day</v>
+      </c>
+      <c r="D60" s="1">
+        <v>0.00004212962962962963</v>
+      </c>
+      <c r="E60" s="1">
+        <v>0.000049074074074074075</v>
       </c>
       <c r="F60" t="str">
-        <v>black screen</v>
+        <v>Speaker 2</v>
       </c>
       <c r="G60" t="str">
-        <v>Vote as if your life depends on it.</v>
+        <v>For our children.</v>
+      </c>
+      <c r="H60">
+        <v>17</v>
       </c>
     </row>
     <row r="61">
       <c r="A61">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C61" t="str">
-        <v>chicken little</v>
-      </c>
-      <c r="D61" t="str">
-        <v>outro</v>
-      </c>
-      <c r="E61" t="str">
-        <v>outro</v>
+        <v>save the day</v>
+      </c>
+      <c r="D61" s="1">
+        <v>0.00005069444444444444</v>
+      </c>
+      <c r="E61" s="1">
+        <v>0.0000587962962962963</v>
       </c>
       <c r="F61" t="str">
-        <v>black screen</v>
+        <v>Speaker 1</v>
       </c>
       <c r="G61" t="str">
-        <v>Vote for Republican [Candidate X] on November 3</v>
+        <v>For our communities.</v>
+      </c>
+      <c r="H61">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62">
+        <v>0</v>
+      </c>
+      <c r="C62" t="str">
+        <v>save the day</v>
+      </c>
+      <c r="D62" s="1">
+        <v>0.0000699074074074074</v>
+      </c>
+      <c r="E62" s="1">
+        <v>0.00007824074074074074</v>
+      </c>
+      <c r="F62" t="str">
+        <v>Speaker 2</v>
+      </c>
+      <c r="G62" t="str">
+        <v>For our communities.</v>
+      </c>
+      <c r="H62">
+        <v>20</v>
       </c>
     </row>
     <row r="63">
       <c r="A63">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C63" t="str">
-        <v>korea rain</v>
-      </c>
-      <c r="D63" t="str">
-        <v>title</v>
-      </c>
-      <c r="E63" t="str">
-        <v>title</v>
+        <v>save the day</v>
+      </c>
+      <c r="D63" s="1">
+        <v>0.00008171296296296296</v>
+      </c>
+      <c r="E63" s="1">
+        <v>0.00009050925925925927</v>
       </c>
       <c r="F63" t="str">
-        <v>meta data</v>
+        <v>Speaker 1</v>
       </c>
       <c r="G63" t="str">
-        <v>Impressed with your leaders?</v>
+        <v>For America.</v>
+      </c>
+      <c r="H63">
+        <v>12</v>
       </c>
     </row>
     <row r="64">
       <c r="A64">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C64" t="str">
-        <v>korea rain</v>
-      </c>
-      <c r="D64" t="str">
-        <v>description</v>
-      </c>
-      <c r="E64" t="str">
-        <v>description</v>
+        <v>save the day</v>
+      </c>
+      <c r="D64" s="1">
+        <v>0.00009212962962962963</v>
+      </c>
+      <c r="E64" s="1">
+        <v>0.00009976851851851851</v>
       </c>
       <c r="F64" t="str">
-        <v>meta data</v>
+        <v>Speaker 1</v>
       </c>
       <c r="G64" t="str">
-        <v>A man tries to impress a woman with an idea for protecting her from the rain. She has the real solution.</v>
+        <v>For America.</v>
+      </c>
+      <c r="H64">
+        <v>12</v>
       </c>
     </row>
     <row r="65">
       <c r="A65">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C65" t="str">
-        <v>korea rain</v>
-      </c>
-      <c r="D65" t="str">
-        <v>intro</v>
-      </c>
-      <c r="E65" t="str">
-        <v>intro</v>
+        <v>save the day</v>
+      </c>
+      <c r="D65" s="1">
+        <v>0.0001011574074074074</v>
+      </c>
+      <c r="E65" s="1">
+        <v>0.00010833333333333333</v>
       </c>
       <c r="F65" t="str">
-        <v>black screen</v>
+        <v>Speaker 2</v>
       </c>
       <c r="G65" t="str">
-        <v>Democrat [CandidateX] wants to impress you.</v>
+        <v>For America.</v>
+      </c>
+      <c r="H65">
+        <v>12</v>
       </c>
     </row>
     <row r="66">
       <c r="A66">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C66" t="str">
-        <v>korea rain</v>
+        <v>save the day</v>
+      </c>
+      <c r="D66" s="1">
+        <v>0.00011921296296296297</v>
+      </c>
+      <c r="E66" s="1">
+        <v>0.00014699074074074075</v>
       </c>
       <c r="F66" t="str">
-        <v>Insert candidates heads. Democrat is man. Republican is woman.</v>
+        <v>Speaker 2</v>
       </c>
       <c r="G66" t="str">
-        <v>Man and woman converse (actual subtitles)</v>
+        <v>All it takes is all of us.</v>
+      </c>
+      <c r="H66">
+        <v>26</v>
       </c>
     </row>
     <row r="67">
       <c r="A67">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C67" t="str">
-        <v>korea rain</v>
-      </c>
-      <c r="D67" t="str">
-        <v>outro</v>
-      </c>
-      <c r="E67" t="str">
-        <v>outro</v>
+        <v>save the day</v>
+      </c>
+      <c r="D67" s="1">
+        <v>0.0001497685185185185</v>
+      </c>
+      <c r="E67" s="1">
+        <v>0.00015486111111111112</v>
       </c>
       <c r="F67" t="str">
-        <v>black screen</v>
+        <v>Speaker 2</v>
       </c>
       <c r="G67" t="str">
-        <v>For real solutions …</v>
+        <v>All of us.</v>
+      </c>
+      <c r="H67">
+        <v>10</v>
       </c>
     </row>
     <row r="68">
       <c r="A68">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C68" t="str">
-        <v>korea rain</v>
-      </c>
-      <c r="D68" t="str">
-        <v>outro</v>
-      </c>
-      <c r="E68" t="str">
-        <v>outro</v>
+        <v>save the day</v>
+      </c>
+      <c r="D68" s="1">
+        <v>0.0001550925925925926</v>
+      </c>
+      <c r="E68" s="1">
+        <v>0.00016319444444444443</v>
       </c>
       <c r="F68" t="str">
-        <v>black screen</v>
+        <v>Speaker 2</v>
       </c>
       <c r="G68" t="str">
-        <v>Vote for Republican [Candidate X] on November 3</v>
+        <v>All of us.</v>
+      </c>
+      <c r="H68">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69">
+        <v>0</v>
+      </c>
+      <c r="C69" t="str">
+        <v>save the day</v>
+      </c>
+      <c r="D69" s="1">
+        <v>0.0001662037037037037</v>
+      </c>
+      <c r="E69" s="1">
+        <v>0.00021111111111111108</v>
+      </c>
+      <c r="F69" t="str">
+        <v>Speaker 1</v>
+      </c>
+      <c r="G69" t="str">
+        <v>We cannot pretend both sides are equally unfavorable.</v>
+      </c>
+      <c r="H69">
+        <v>53</v>
       </c>
     </row>
     <row r="70">
@@ -1613,19 +1746,22 @@
         <v>0</v>
       </c>
       <c r="C70" t="str">
-        <v>cheeseburger fail</v>
-      </c>
-      <c r="D70" t="str">
-        <v>title</v>
-      </c>
-      <c r="E70" t="str">
-        <v>title</v>
+        <v>save the day</v>
+      </c>
+      <c r="D70" s="1">
+        <v>0.0002122685185185185</v>
+      </c>
+      <c r="E70" s="1">
+        <v>0.00023240740740740738</v>
       </c>
       <c r="F70" t="str">
-        <v>meta data</v>
+        <v>Speaker 2</v>
       </c>
       <c r="G70" t="str">
-        <v>Losing patience with your leaders?</v>
+        <v>We can't say one vote doesn't matter.</v>
+      </c>
+      <c r="H70">
+        <v>37</v>
       </c>
     </row>
     <row r="71">
@@ -1633,19 +1769,22 @@
         <v>0</v>
       </c>
       <c r="C71" t="str">
-        <v>cheeseburger fail</v>
-      </c>
-      <c r="D71" t="str">
-        <v>description</v>
-      </c>
-      <c r="E71" t="str">
-        <v>description</v>
+        <v>save the day</v>
+      </c>
+      <c r="D71" s="1">
+        <v>0.00023333333333333333</v>
+      </c>
+      <c r="E71" s="1">
+        <v>0.00024236111111111114</v>
       </c>
       <c r="F71" t="str">
-        <v>meta data</v>
+        <v>Speaker 1</v>
       </c>
       <c r="G71" t="str">
-        <v>A fast food customer, representing voters, is finally fed up with the service he has received.</v>
+        <v>Your vote matters.</v>
+      </c>
+      <c r="H71">
+        <v>18</v>
       </c>
     </row>
     <row r="72">
@@ -1653,19 +1792,22 @@
         <v>0</v>
       </c>
       <c r="C72" t="str">
-        <v>cheeseburger fail</v>
-      </c>
-      <c r="D72" t="str">
-        <v>intro</v>
-      </c>
-      <c r="E72" t="str">
-        <v>intro</v>
+        <v>save the day</v>
+      </c>
+      <c r="D72" s="1">
+        <v>0.00024398148148148147</v>
+      </c>
+      <c r="E72" s="1">
+        <v>0.0002546296296296296</v>
       </c>
       <c r="F72" t="str">
-        <v>black screen</v>
+        <v>Speaker 2</v>
       </c>
       <c r="G72" t="str">
-        <v>[CandidateX] feels your pain.</v>
+        <v>Your vote matters.</v>
+      </c>
+      <c r="H72">
+        <v>18</v>
       </c>
     </row>
     <row r="73">
@@ -1673,16 +1815,22 @@
         <v>0</v>
       </c>
       <c r="C73" t="str">
-        <v>cheeseburger fail</v>
-      </c>
-      <c r="D73" t="str">
-        <v>:00</v>
-      </c>
-      <c r="E73" t="str">
-        <v>:31</v>
+        <v>save the day</v>
+      </c>
+      <c r="D73" s="1">
+        <v>0.0002564814814814815</v>
+      </c>
+      <c r="E73" s="1">
+        <v>0.0002666666666666667</v>
+      </c>
+      <c r="F73" t="str">
+        <v>Speaker 2</v>
       </c>
       <c r="G73" t="str">
-        <v>Man complains at fast food window</v>
+        <v>It affects everything.</v>
+      </c>
+      <c r="H73">
+        <v>22</v>
       </c>
     </row>
     <row r="74">
@@ -1690,19 +1838,22 @@
         <v>0</v>
       </c>
       <c r="C74" t="str">
-        <v>cheeseburger fail</v>
-      </c>
-      <c r="D74" t="str">
-        <v>outro</v>
-      </c>
-      <c r="E74" t="str">
-        <v>outro</v>
+        <v>save the day</v>
+      </c>
+      <c r="D74" s="1">
+        <v>0.00026828703703703704</v>
+      </c>
+      <c r="E74" s="1">
+        <v>0.0002863425925925926</v>
       </c>
       <c r="F74" t="str">
-        <v>black screen</v>
+        <v>Speaker 1</v>
       </c>
       <c r="G74" t="str">
-        <v>For competence you can count on …</v>
+        <v>See, this isn't just an election.</v>
+      </c>
+      <c r="H74">
+        <v>33</v>
       </c>
     </row>
     <row r="75">
@@ -1710,24 +1861,988 @@
         <v>0</v>
       </c>
       <c r="C75" t="str">
+        <v>save the day</v>
+      </c>
+      <c r="D75" s="1">
+        <v>0.0002895833333333333</v>
+      </c>
+      <c r="E75" s="1">
+        <v>0.0003018518518518518</v>
+      </c>
+      <c r="F75" t="str">
+        <v>Speaker 1</v>
+      </c>
+      <c r="G75" t="str">
+        <v>It's a tipping point.</v>
+      </c>
+      <c r="H75">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76">
+        <v>0</v>
+      </c>
+      <c r="C76" t="str">
+        <v>save the day</v>
+      </c>
+      <c r="D76" s="1">
+        <v>0.0003039351851851852</v>
+      </c>
+      <c r="E76" s="1">
+        <v>0.0003104166666666667</v>
+      </c>
+      <c r="F76" t="str">
+        <v>Speaker 2</v>
+      </c>
+      <c r="G76" t="str">
+        <v>For the country.</v>
+      </c>
+      <c r="H76">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77">
+        <v>0</v>
+      </c>
+      <c r="C77" t="str">
+        <v>save the day</v>
+      </c>
+      <c r="D77" s="1">
+        <v>0.00031319444444444445</v>
+      </c>
+      <c r="E77" s="1">
+        <v>0.00032175925925925926</v>
+      </c>
+      <c r="F77" t="str">
+        <v>Speaker 1</v>
+      </c>
+      <c r="G77" t="str">
+        <v>For the world.</v>
+      </c>
+      <c r="H77">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78">
+        <v>0</v>
+      </c>
+      <c r="C78" t="str">
+        <v>save the day</v>
+      </c>
+      <c r="D78" s="1">
+        <v>0.000324537037037037</v>
+      </c>
+      <c r="E78" s="1">
+        <v>0.00033194444444444444</v>
+      </c>
+      <c r="F78" t="str">
+        <v>Speaker 1</v>
+      </c>
+      <c r="G78" t="str">
+        <v>For your world.</v>
+      </c>
+      <c r="H78">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79">
+        <v>0</v>
+      </c>
+      <c r="C79" t="str">
+        <v>save the day</v>
+      </c>
+      <c r="D79" t="str">
+        <v>outro</v>
+      </c>
+      <c r="E79" t="str">
+        <v>outro</v>
+      </c>
+      <c r="F79" t="str">
+        <v>black screen</v>
+      </c>
+      <c r="G79" t="str">
+        <v>There's at least one thing we can agree on ...</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80">
+        <v>0</v>
+      </c>
+      <c r="C80" t="str">
+        <v>save the day</v>
+      </c>
+      <c r="D80" t="str">
+        <v>outro</v>
+      </c>
+      <c r="E80" t="str">
+        <v>outro</v>
+      </c>
+      <c r="F80" t="str">
+        <v>black screen</v>
+      </c>
+      <c r="G80" t="str">
+        <v>"We cannot pretend both sides are equally unfavorable."</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81">
+        <v>0</v>
+      </c>
+      <c r="C81" t="str">
+        <v>save the day</v>
+      </c>
+      <c r="D81" t="str">
+        <v>outro</v>
+      </c>
+      <c r="E81" t="str">
+        <v>outro</v>
+      </c>
+      <c r="F81" t="str">
+        <v>black screen</v>
+      </c>
+      <c r="G81" t="str">
+        <v>Vote for Republican [Candidate X] on November 3</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83">
+        <v>0</v>
+      </c>
+      <c r="C83" t="str">
+        <v>chicken little</v>
+      </c>
+      <c r="D83" t="str">
+        <v>title</v>
+      </c>
+      <c r="E83" t="str">
+        <v>title</v>
+      </c>
+      <c r="F83" t="str">
+        <v>meta data</v>
+      </c>
+      <c r="G83" t="str">
+        <v>The new star of the Democratic Party looks familiar</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84">
+        <v>3</v>
+      </c>
+      <c r="C84" t="str">
+        <v>chicken little</v>
+      </c>
+      <c r="D84" t="str">
+        <v>description</v>
+      </c>
+      <c r="E84" t="str">
+        <v>description</v>
+      </c>
+      <c r="F84" t="str">
+        <v>meta data</v>
+      </c>
+      <c r="G84" t="str">
+        <v>Border walls are useless when the enemy is within, as these clips from the 1943 Disney cartoon Chicken Little illustrate.</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85">
+        <v>0</v>
+      </c>
+      <c r="C85" t="str">
+        <v>chicken little</v>
+      </c>
+      <c r="D85" s="1">
+        <v>0.000019791666666666665</v>
+      </c>
+      <c r="E85" s="1">
+        <v>0.00018020833333333333</v>
+      </c>
+      <c r="F85" t="str">
+        <v>Speaker 1</v>
+      </c>
+      <c r="G85" t="str">
+        <v>Our story takes place in a nice cozy little farmyard as our story continues We find all our fine-feathered friends happy and contented and why not didn't they have a big strong fence protecting them?</v>
+      </c>
+      <c r="H85">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86">
+        <v>0</v>
+      </c>
+      <c r="C86" t="str">
+        <v>chicken little</v>
+      </c>
+      <c r="D86" s="1">
+        <v>0.00018622685185185186</v>
+      </c>
+      <c r="E86" s="1">
+        <v>0.00019618055555555553</v>
+      </c>
+      <c r="F86" t="str">
+        <v>Speaker 2</v>
+      </c>
+      <c r="G86" t="str">
+        <v>But wait a minute.</v>
+      </c>
+      <c r="H86">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87">
+        <v>0</v>
+      </c>
+      <c r="C87" t="str">
+        <v>chicken little</v>
+      </c>
+      <c r="D87" s="1">
+        <v>0.00020289351851851854</v>
+      </c>
+      <c r="E87" s="1">
+        <v>0.0002119212962962963</v>
+      </c>
+      <c r="F87" t="str">
+        <v>Speaker 1</v>
+      </c>
+      <c r="G87" t="str">
+        <v>What's this?</v>
+      </c>
+      <c r="H87">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88">
+        <v>0</v>
+      </c>
+      <c r="C88" t="str">
+        <v>chicken little</v>
+      </c>
+      <c r="D88" s="1">
+        <v>0.0002643518518518518</v>
+      </c>
+      <c r="E88" s="1">
+        <v>0.0003881944444444444</v>
+      </c>
+      <c r="F88" t="str">
+        <v>Speaker 1</v>
+      </c>
+      <c r="G88" t="str">
+        <v>It's foxy loxy the poultry fancier Looks like he's taken an interest in our little community a culinary interest So why doesn't he just jump in and help himself?</v>
+      </c>
+      <c r="H88">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89">
+        <v>0</v>
+      </c>
+      <c r="C89" t="str">
+        <v>chicken little</v>
+      </c>
+      <c r="D89" s="1">
+        <v>0.0003881944444444444</v>
+      </c>
+      <c r="E89" s="1">
+        <v>0.0004817129629629629</v>
+      </c>
+      <c r="F89" t="str">
+        <v>Speaker 1</v>
+      </c>
+      <c r="G89" t="str">
+        <v>Do you suppose it's because of the high fence or the locks on the inside or the farmers shotgun?</v>
+      </c>
+      <c r="H89">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90">
+        <v>0</v>
+      </c>
+      <c r="C90" t="str">
+        <v>chicken little</v>
+      </c>
+      <c r="D90" s="1">
+        <v>0.0004974537037037036</v>
+      </c>
+      <c r="E90" s="1">
+        <v>0.0006237268518518519</v>
+      </c>
+      <c r="F90" t="str">
+        <v>Speaker 1</v>
+      </c>
+      <c r="G90" t="str">
+        <v>But I'm not a fox for nothing besides there's more than one way to plug a chicken Psychology why should I just get one when I can get them all?</v>
+      </c>
+      <c r="H90">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91">
+        <v>0</v>
+      </c>
+      <c r="C91" t="str">
+        <v>chicken little</v>
+      </c>
+      <c r="D91" s="1">
+        <v>0.0006393518518518519</v>
+      </c>
+      <c r="E91" s="1">
+        <v>0.0006939814814814815</v>
+      </c>
+      <c r="F91" t="str">
+        <v>Speaker 1</v>
+      </c>
+      <c r="G91" t="str">
+        <v>Quote to influence the masses aim first at the least intelligent unquote</v>
+      </c>
+      <c r="H91">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92">
+        <v>3</v>
+      </c>
+      <c r="C92" t="str">
+        <v>chicken little</v>
+      </c>
+      <c r="D92" t="str">
+        <v>outro</v>
+      </c>
+      <c r="E92" t="str">
+        <v>outro</v>
+      </c>
+      <c r="F92" t="str">
+        <v>black screen</v>
+      </c>
+      <c r="G92" t="str">
+        <v>Vote as if your life depends on it.</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93">
+        <v>3</v>
+      </c>
+      <c r="C93" t="str">
+        <v>chicken little</v>
+      </c>
+      <c r="D93" t="str">
+        <v>outro</v>
+      </c>
+      <c r="E93" t="str">
+        <v>outro</v>
+      </c>
+      <c r="F93" t="str">
+        <v>black screen</v>
+      </c>
+      <c r="G93" t="str">
+        <v>Vote for Republican [Candidate X] on November 3</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95">
+        <v>3</v>
+      </c>
+      <c r="C95" t="str">
+        <v>korea rain</v>
+      </c>
+      <c r="D95" t="str">
+        <v>title</v>
+      </c>
+      <c r="E95" t="str">
+        <v>title</v>
+      </c>
+      <c r="F95" t="str">
+        <v>meta data</v>
+      </c>
+      <c r="G95" t="str">
+        <v>Impressed with your leaders?</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96">
+        <v>3</v>
+      </c>
+      <c r="C96" t="str">
+        <v>korea rain</v>
+      </c>
+      <c r="D96" t="str">
+        <v>description</v>
+      </c>
+      <c r="E96" t="str">
+        <v>description</v>
+      </c>
+      <c r="F96" t="str">
+        <v>meta data</v>
+      </c>
+      <c r="G96" t="str">
+        <v>A man tries to impress a woman with an idea for protecting her from the rain. She has the real solution.</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97">
+        <v>3</v>
+      </c>
+      <c r="C97" t="str">
+        <v>korea rain</v>
+      </c>
+      <c r="D97" t="str">
+        <v>intro</v>
+      </c>
+      <c r="E97" t="str">
+        <v>intro</v>
+      </c>
+      <c r="F97" t="str">
+        <v>black screen</v>
+      </c>
+      <c r="G97" t="str">
+        <v>Democrat [CandidateX] wants to impress you.</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98">
+        <v>3</v>
+      </c>
+      <c r="C98" t="str">
+        <v>korea rain</v>
+      </c>
+      <c r="D98" s="1">
+        <v>0.000013541666666666666</v>
+      </c>
+      <c r="E98" s="1">
+        <v>0.000023495370370370367</v>
+      </c>
+      <c r="F98" t="str">
+        <v>Speaker 1</v>
+      </c>
+      <c r="G98" t="str">
+        <v>Why is it raining all of a sudden?</v>
+      </c>
+      <c r="H98">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99">
+        <v>3</v>
+      </c>
+      <c r="C99" t="str">
+        <v>korea rain</v>
+      </c>
+      <c r="D99" s="1">
+        <v>0.000028587962962962966</v>
+      </c>
+      <c r="E99" s="1">
+        <v>0.000041782407407407405</v>
+      </c>
+      <c r="F99" t="str">
+        <v>Speaker 1</v>
+      </c>
+      <c r="G99" t="str">
+        <v>There wasn't any forecast today.</v>
+      </c>
+      <c r="H99">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100">
+        <v>3</v>
+      </c>
+      <c r="C100" t="str">
+        <v>korea rain</v>
+      </c>
+      <c r="D100" s="1">
+        <v>0.00004479166666666667</v>
+      </c>
+      <c r="E100" s="1">
+        <v>0.00004756944444444445</v>
+      </c>
+      <c r="F100" t="str">
+        <v>Speaker 2</v>
+      </c>
+      <c r="G100" t="str">
+        <v>I know.</v>
+      </c>
+      <c r="H100">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101">
+        <v>3</v>
+      </c>
+      <c r="C101" t="str">
+        <v>korea rain</v>
+      </c>
+      <c r="D101" s="1">
+        <v>0.000060532407407407414</v>
+      </c>
+      <c r="E101" s="1">
+        <v>0.00006840277777777778</v>
+      </c>
+      <c r="F101" t="str">
+        <v>Speaker 1</v>
+      </c>
+      <c r="G101" t="str">
+        <v>Why is it raining all of a sudden?</v>
+      </c>
+      <c r="H101">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102">
+        <v>3</v>
+      </c>
+      <c r="C102" t="str">
+        <v>korea rain</v>
+      </c>
+      <c r="D102" s="1">
+        <v>0.00008229166666666667</v>
+      </c>
+      <c r="E102" s="1">
+        <v>0.00018703703703703704</v>
+      </c>
+      <c r="F102" t="str">
+        <v>Speaker 1</v>
+      </c>
+      <c r="G102" t="str">
+        <v>Should we run together?</v>
+      </c>
+      <c r="H102">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103">
+        <v>3</v>
+      </c>
+      <c r="C103" t="str">
+        <v>korea rain</v>
+      </c>
+      <c r="D103" s="1">
+        <v>0.00019212962962962963</v>
+      </c>
+      <c r="E103" s="1">
+        <v>0.00020555555555555559</v>
+      </c>
+      <c r="F103" t="str">
+        <v>Speaker 2</v>
+      </c>
+      <c r="G103" t="str">
+        <v>We shouldn't run together.</v>
+      </c>
+      <c r="H103">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104">
+        <v>3</v>
+      </c>
+      <c r="C104" t="str">
+        <v>korea rain</v>
+      </c>
+      <c r="D104" s="1">
+        <v>0.00021319444444444446</v>
+      </c>
+      <c r="E104" s="1">
+        <v>0.00021666666666666666</v>
+      </c>
+      <c r="F104" t="str">
+        <v>Speaker 2</v>
+      </c>
+      <c r="G104" t="str">
+        <v>Okay.</v>
+      </c>
+      <c r="H104">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105">
+        <v>3</v>
+      </c>
+      <c r="C105" t="str">
+        <v>korea rain</v>
+      </c>
+      <c r="D105" t="str">
+        <v>outro</v>
+      </c>
+      <c r="E105" t="str">
+        <v>outro</v>
+      </c>
+      <c r="F105" t="str">
+        <v>black screen</v>
+      </c>
+      <c r="G105" t="str">
+        <v>For real solutions …</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106">
+        <v>3</v>
+      </c>
+      <c r="C106" t="str">
+        <v>korea rain</v>
+      </c>
+      <c r="D106" t="str">
+        <v>outro</v>
+      </c>
+      <c r="E106" t="str">
+        <v>outro</v>
+      </c>
+      <c r="F106" t="str">
+        <v>black screen</v>
+      </c>
+      <c r="G106" t="str">
+        <v>Vote for Republican [Candidate X] on November 3</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108">
+        <v>0</v>
+      </c>
+      <c r="C108" t="str">
         <v>cheeseburger fail</v>
       </c>
-      <c r="D75" t="str">
-        <v>outro</v>
-      </c>
-      <c r="E75" t="str">
-        <v>outro</v>
-      </c>
-      <c r="F75" t="str">
+      <c r="D108" t="str">
+        <v>title</v>
+      </c>
+      <c r="E108" t="str">
+        <v>title</v>
+      </c>
+      <c r="F108" t="str">
+        <v>meta data</v>
+      </c>
+      <c r="G108" t="str">
+        <v>Losing patience with your leaders?</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109">
+        <v>0</v>
+      </c>
+      <c r="C109" t="str">
+        <v>cheeseburger fail</v>
+      </c>
+      <c r="D109" t="str">
+        <v>description</v>
+      </c>
+      <c r="E109" t="str">
+        <v>description</v>
+      </c>
+      <c r="F109" t="str">
+        <v>meta data</v>
+      </c>
+      <c r="G109" t="str">
+        <v>A fast food customer, representing voters, is finally fed up with the service he has received.</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110">
+        <v>0</v>
+      </c>
+      <c r="C110" t="str">
+        <v>cheeseburger fail</v>
+      </c>
+      <c r="D110" t="str">
+        <v>intro</v>
+      </c>
+      <c r="E110" t="str">
+        <v>intro</v>
+      </c>
+      <c r="F110" t="str">
         <v>black screen</v>
       </c>
-      <c r="G75" t="str">
+      <c r="G110" t="str">
+        <v>[CandidateX] feels your pain.</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111">
+        <v>0</v>
+      </c>
+      <c r="C111" t="str">
+        <v>cheeseburger fail</v>
+      </c>
+      <c r="D111" s="1">
+        <v>0</v>
+      </c>
+      <c r="E111" s="1">
+        <v>0.00002962962962962963</v>
+      </c>
+      <c r="F111" t="str">
+        <v>Speaker 1</v>
+      </c>
+      <c r="G111" t="str">
+        <v>When you have a cheeseburger, you have a cheeseburger.</v>
+      </c>
+      <c r="H111">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112">
+        <v>0</v>
+      </c>
+      <c r="C112" t="str">
+        <v>cheeseburger fail</v>
+      </c>
+      <c r="D112" s="1">
+        <v>0.00003263888888888889</v>
+      </c>
+      <c r="E112" s="1">
+        <v>0.00005092592592592593</v>
+      </c>
+      <c r="F112" t="str">
+        <v>Speaker 1</v>
+      </c>
+      <c r="G112" t="str">
+        <v>If you have hamburger, you have hamburger.</v>
+      </c>
+      <c r="H112">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113">
+        <v>0</v>
+      </c>
+      <c r="C113" t="str">
+        <v>cheeseburger fail</v>
+      </c>
+      <c r="D113" s="1">
+        <v>0.00006157407407407408</v>
+      </c>
+      <c r="E113" s="1">
+        <v>0.0001076388888888889</v>
+      </c>
+      <c r="F113" t="str">
+        <v>Speaker 2</v>
+      </c>
+      <c r="G113" t="str">
+        <v>I want my money back, I want my money back now, and I want it fast.</v>
+      </c>
+      <c r="H113">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114">
+        <v>0</v>
+      </c>
+      <c r="C114" t="str">
+        <v>cheeseburger fail</v>
+      </c>
+      <c r="D114" s="1">
+        <v>0.00010972222222222222</v>
+      </c>
+      <c r="E114" s="1">
+        <v>0.00015162037037037037</v>
+      </c>
+      <c r="F114" t="str">
+        <v>Speaker 2</v>
+      </c>
+      <c r="G114" t="str">
+        <v>There's not even bacon on this and not onion on this and not anything that I asked for.</v>
+      </c>
+      <c r="H114">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115">
+        <v>0</v>
+      </c>
+      <c r="C115" t="str">
+        <v>cheeseburger fail</v>
+      </c>
+      <c r="D115" s="1">
+        <v>0.00015717592592592592</v>
+      </c>
+      <c r="E115" s="1">
+        <v>0.00018217592592592593</v>
+      </c>
+      <c r="F115" t="str">
+        <v>Speaker 2</v>
+      </c>
+      <c r="G115" t="str">
+        <v>This is such incompetence, I cannot believe it.</v>
+      </c>
+      <c r="H115">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116">
+        <v>0</v>
+      </c>
+      <c r="C116" t="str">
+        <v>cheeseburger fail</v>
+      </c>
+      <c r="D116" s="1">
+        <v>0.0001837962962962963</v>
+      </c>
+      <c r="E116" s="1">
+        <v>0.0002016203703703704</v>
+      </c>
+      <c r="F116" t="str">
+        <v>Speaker 2</v>
+      </c>
+      <c r="G116" t="str">
+        <v>It happens every time I come here.</v>
+      </c>
+      <c r="H116">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117">
+        <v>0</v>
+      </c>
+      <c r="C117" t="str">
+        <v>cheeseburger fail</v>
+      </c>
+      <c r="D117" s="1">
+        <v>0.00020509259259259257</v>
+      </c>
+      <c r="E117" s="1">
+        <v>0.0002622685185185185</v>
+      </c>
+      <c r="F117" t="str">
+        <v>Speaker 2</v>
+      </c>
+      <c r="G117" t="str">
+        <v>I'm losing my s*** because this happened the past three times I've come.</v>
+      </c>
+      <c r="H117">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118">
+        <v>0</v>
+      </c>
+      <c r="C118" t="str">
+        <v>cheeseburger fail</v>
+      </c>
+      <c r="D118" s="1">
+        <v>0.0002696759259259259</v>
+      </c>
+      <c r="E118" s="1">
+        <v>0.00030138888888888885</v>
+      </c>
+      <c r="F118" t="str">
+        <v>Speaker 2</v>
+      </c>
+      <c r="G118" t="str">
+        <v>Please be competent once in your life.</v>
+      </c>
+      <c r="H118">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119">
+        <v>0</v>
+      </c>
+      <c r="C119" t="str">
+        <v>cheeseburger fail</v>
+      </c>
+      <c r="D119" s="1">
+        <v>0.00030902777777777775</v>
+      </c>
+      <c r="E119" s="1">
+        <v>0.00031435185185185185</v>
+      </c>
+      <c r="F119" t="str">
+        <v>Speaker 2</v>
+      </c>
+      <c r="G119" t="str">
+        <v>Once.</v>
+      </c>
+      <c r="H119">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120">
+        <v>0</v>
+      </c>
+      <c r="C120" t="str">
+        <v>cheeseburger fail</v>
+      </c>
+      <c r="D120" s="1">
+        <v>0.0003212962962962963</v>
+      </c>
+      <c r="E120" s="1">
+        <v>0.00034166666666666666</v>
+      </c>
+      <c r="F120" t="str">
+        <v>Speaker 2</v>
+      </c>
+      <c r="G120" t="str">
+        <v>Take an order and fill it.</v>
+      </c>
+      <c r="H120">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121">
+        <v>0</v>
+      </c>
+      <c r="C121" t="str">
+        <v>cheeseburger fail</v>
+      </c>
+      <c r="D121" t="str">
+        <v>outro</v>
+      </c>
+      <c r="E121" t="str">
+        <v>outro</v>
+      </c>
+      <c r="F121" t="str">
+        <v>black screen</v>
+      </c>
+      <c r="G121" t="str">
+        <v>For competence you can count on …</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122">
+        <v>0</v>
+      </c>
+      <c r="C122" t="str">
+        <v>cheeseburger fail</v>
+      </c>
+      <c r="D122" t="str">
+        <v>outro</v>
+      </c>
+      <c r="E122" t="str">
+        <v>outro</v>
+      </c>
+      <c r="F122" t="str">
+        <v>black screen</v>
+      </c>
+      <c r="G122" t="str">
         <v>Vote for Republican [Candidate X] on November 3</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K76"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K123"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>